<commit_message>
Revert "Storys 2 Update"
This reverts commit 96393b7f287998ccc4bd47bb8b4e5152221870b3.
</commit_message>
<xml_diff>
--- a/assets/stories/the_last_prank_of_tomist/story.xlsx
+++ b/assets/stories/the_last_prank_of_tomist/story.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Models And Textures And Rigs\Assets\2025\Graphic\Realistic\Art\PortFolio Website\Versions\Website v10\assets\stories\the_last_prank_of_tomist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A45D9CF-3830-4684-9F9D-985E7115C33E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA69064-C4D2-49CF-82B3-0B23A2504E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{519ED677-905E-4654-B2E6-32D98CCB5F18}"/>
+    <workbookView xWindow="3072" yWindow="3072" windowWidth="30960" windowHeight="12120" xr2:uid="{519ED677-905E-4654-B2E6-32D98CCB5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Genres</t>
   </si>
@@ -384,15 +384,6 @@
 Grace nodded, watching Tomist leap over a pile of rubble. “I always wondered what your imaginary friend looked like, Leo. And now I know. Monkey-man.”
 Leo grinned. “Still mischievous, too.”
 Grace smiled knowingly. “When you were little, if Tomist w</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Leo, a kid who survives a car crash into an alien spaceship, wakes up to find his imaginary friends coming to life.</t>
-  </si>
-  <si>
-    <t>Kids</t>
   </si>
 </sst>
 </file>
@@ -782,9 +773,6 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -792,9 +780,6 @@
       </c>
       <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -817,11 +802,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="9" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
         <v>8</v>

</xml_diff>